<commit_message>
B12-010: fix Dashboard/helper number formats found by a real Excel recalc
Cycle 101 verified the shipped workbook in Excel 16.0 (build 19127) instead of
only re-deriving the rules in Python. The computed values all matched, but the
recalculation exposed seven wrong number formats: a count shown as 100%, the
award rate as $1, requested money as 3000000%, a count as 1900-01-01, the next
deadline as 46328, and the open-deadline helper as a raw serial.

- align Dashboard B6/B7/B8/B9/B10/B12/B13 formats with what each cell shows
- format Opportunities column V as a date inside the formula loop
- add a format regression test (values alone could not catch this)
- record the native recalculation in NATIVE_RECALC_EXCEL_2026-10-19.json
- add the gate method, release baseline and test evidence records
- propagate the new workbook hash (38,765 B / df49ceca) to the manifest, QA
  facts, listing package and tests

Not published. No authorization exists; FACTORY_LIVE_PUBLISH unchanged.
</commit_message>
<xml_diff>
--- a/books/batch12/B12-010_grant_pipeline_tracker.xlsx
+++ b/books/batch12/B12-010_grant_pipeline_tracker.xlsx
@@ -119,7 +119,7 @@
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -6652,7 +6652,7 @@
           <t>Awarded (count)</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="7">
         <f>COUNTIF(Opportunities!$I$2:$I$41,"Awarded")</f>
         <v/>
       </c>
@@ -6668,7 +6668,7 @@
           <t>Award rate</t>
         </is>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="13">
         <f>IFERROR(B6/B5,"")</f>
         <v/>
       </c>
@@ -6700,7 +6700,7 @@
           <t>Total requested (USD)</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="14">
         <f>SUM(Budget!$C$2:$C$121)</f>
         <v/>
       </c>
@@ -6716,7 +6716,7 @@
           <t>Awarded against requested</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="13">
         <f>IF(B9=0,"",B8/B9)</f>
         <v/>
       </c>
@@ -6748,7 +6748,7 @@
           <t>Deadlines due within 14 days</t>
         </is>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="7">
         <f>COUNTIF(Opportunities!$S$2:$S$41,"DUE IN*")</f>
         <v/>
       </c>
@@ -6764,7 +6764,7 @@
           <t>Next deadline (open rows only)</t>
         </is>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="12">
         <f>IF(COUNT(Opportunities!$V$2:$V$41)=0,"",MIN(Opportunities!$V$2:$V$41))</f>
         <v/>
       </c>
@@ -6844,7 +6844,7 @@
           <t>Post-award reports due within 30 days</t>
         </is>
       </c>
-      <c r="B18" s="6">
+      <c r="B18" s="7">
         <f>COUNTIF(Timeline!$F$2:$F$61,"DUE IN*")</f>
         <v/>
       </c>

</xml_diff>